<commit_message>
Add EM-DAT multi-hazard covariates: cyclone + drought GAMs, feature set v7.4 (v0.65.0)
New wind-led tropical-cyclone GAM (impute_cyclone_probability) and
SPEI/precip-led drought GAM (impute_drought_probability), each modeling
their EM-DAT hazard channel with a mechanistically distinct predictor set
rather than folding everything into the precipitation flood label (which
had dropped all tropical-cyclone/surge events). process_EMDAT_data now
emits the cyclone channel alongside floods; feature_sets gains the v7.4
hazard feature set (MINFEAT_V7_4); globals registers the new covariate
names. Unit tests for both GAMs, the GAM train/stop leakage guard, and the
updated EM-DAT panel; synthetic EM-DAT fixture refreshed with cyclone rows.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/testthat/fixtures/public_emdat_2099-01-01_synthetic.xlsx
+++ b/tests/testthat/fixtures/public_emdat_2099-01-01_synthetic.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="EM-DAT Data" sheetId="1" r:id="rId1"/>
-    <sheet name="EM-DAT Info" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -352,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -368,45 +367,50 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Disaster Subtype</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>ISO</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Start Year</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Start Month</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Start Day</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>End Year</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>End Month</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>End Day</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Total Deaths</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Total Affected</t>
         </is>
@@ -423,33 +427,33 @@
           <t>Epidemic</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>KEN</t>
         </is>
       </c>
-      <c r="D2">
-        <v>2015</v>
-      </c>
       <c r="E2">
+        <v>2015</v>
+      </c>
+      <c r="F2">
         <v>6</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>1</v>
       </c>
-      <c r="G2">
-        <v>2015</v>
-      </c>
       <c r="H2">
+        <v>2015</v>
+      </c>
+      <c r="I2">
         <v>6</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>30</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>99</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>999</v>
       </c>
     </row>
@@ -464,33 +468,33 @@
           <t>Flood</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D3">
-        <v>2015</v>
-      </c>
       <c r="E3">
-        <v>5</v>
+        <v>2015</v>
       </c>
       <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
         <v>10</v>
       </c>
-      <c r="G3">
-        <v>2015</v>
-      </c>
       <c r="H3">
-        <v>5</v>
+        <v>2015</v>
       </c>
       <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3">
         <v>20</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>0</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>999</v>
       </c>
     </row>
@@ -505,33 +509,33 @@
           <t>Flood</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>KEN</t>
         </is>
       </c>
-      <c r="D4">
-        <v>2015</v>
-      </c>
       <c r="E4">
-        <v>5</v>
+        <v>2015</v>
       </c>
       <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4">
         <v>4</v>
       </c>
-      <c r="G4">
-        <v>2015</v>
-      </c>
       <c r="H4">
-        <v>5</v>
+        <v>2015</v>
       </c>
       <c r="I4">
+        <v>5</v>
+      </c>
+      <c r="J4">
         <v>4</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>2</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>100</v>
       </c>
     </row>
@@ -546,33 +550,33 @@
           <t>Flood</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>KEN</t>
         </is>
       </c>
-      <c r="D5">
-        <v>2015</v>
-      </c>
       <c r="E5">
-        <v>5</v>
+        <v>2015</v>
       </c>
       <c r="F5">
         <v>5</v>
       </c>
       <c r="G5">
-        <v>2015</v>
+        <v>5</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>2015</v>
       </c>
       <c r="I5">
         <v>5</v>
       </c>
       <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
         <v>8</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>300</v>
       </c>
     </row>
@@ -587,33 +591,33 @@
           <t>Flood</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>NGA</t>
         </is>
       </c>
-      <c r="D6">
-        <v>2015</v>
-      </c>
       <c r="E6">
-        <v>5</v>
+        <v>2015</v>
       </c>
       <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
         <v>4</v>
       </c>
-      <c r="G6">
-        <v>2015</v>
-      </c>
       <c r="H6">
-        <v>5</v>
+        <v>2015</v>
       </c>
       <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
         <v>24</v>
       </c>
-      <c r="J6">
-        <v>5</v>
-      </c>
       <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
         <v>1000</v>
       </c>
     </row>
@@ -628,27 +632,27 @@
           <t>Flood</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>UGA</t>
         </is>
       </c>
-      <c r="D7">
-        <v>2015</v>
-      </c>
       <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="G7">
-        <v>2015</v>
+        <v>2015</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
       </c>
       <c r="H7">
-        <v>5</v>
-      </c>
-      <c r="J7">
+        <v>2015</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+      <c r="K7">
         <v>0</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>50</v>
       </c>
     </row>
@@ -663,68 +667,264 @@
           <t>Flood</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>MOZ</t>
         </is>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>2010</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>3</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>15</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>2010</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>3</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>15</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>0</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>200</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Synthetic</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Built for unit tests</t>
-        </is>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2020-0001-MOZ-cyc</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tropical cyclone</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MOZ</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>2020</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>20</v>
+      </c>
+      <c r="H9">
+        <v>2020</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>26</v>
+      </c>
+      <c r="K9">
+        <v>50</v>
+      </c>
+      <c r="L9">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2021-0001-ZWE-surge</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Storm surge</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="E10">
+        <v>2021</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10">
+        <v>8</v>
+      </c>
+      <c r="H10">
+        <v>2021</v>
+      </c>
+      <c r="I10">
+        <v>2</v>
+      </c>
+      <c r="J10">
+        <v>14</v>
+      </c>
+      <c r="K10">
+        <v>10</v>
+      </c>
+      <c r="L10">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2020-0002-NGA-stormgen</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Storm (General)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NGA</t>
+        </is>
+      </c>
+      <c r="E11">
+        <v>2020</v>
+      </c>
+      <c r="F11">
+        <v>6</v>
+      </c>
+      <c r="G11">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>2020</v>
+      </c>
+      <c r="I11">
+        <v>6</v>
+      </c>
+      <c r="J11">
+        <v>12</v>
+      </c>
+      <c r="K11">
+        <v>3</v>
+      </c>
+      <c r="L11">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2020-0003-KEN-severe</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Severe weather</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>KEN</t>
+        </is>
+      </c>
+      <c r="E12">
+        <v>2020</v>
+      </c>
+      <c r="F12">
+        <v>7</v>
+      </c>
+      <c r="G12">
+        <v>10</v>
+      </c>
+      <c r="H12">
+        <v>2020</v>
+      </c>
+      <c r="I12">
+        <v>7</v>
+      </c>
+      <c r="J12">
+        <v>12</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2020-0004-MWI-light</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Storm</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lightning/Thunderstorms</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MWI</t>
+        </is>
+      </c>
+      <c r="E13">
+        <v>2020</v>
+      </c>
+      <c r="F13">
+        <v>8</v>
+      </c>
+      <c r="G13">
+        <v>10</v>
+      </c>
+      <c r="H13">
+        <v>2020</v>
+      </c>
+      <c r="I13">
+        <v>8</v>
+      </c>
+      <c r="J13">
+        <v>12</v>
+      </c>
+      <c r="K13">
+        <v>2</v>
+      </c>
+      <c r="L13">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>